<commit_message>
them cot ghi chu duc
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/PKH_BOF.xlsx
+++ b/dataproduct.api/wwwroot/templates/PKH_BOF.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246CCE11-0C59-4EBE-9B58-39EDA360DED9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D3BDCA3-1644-4D0C-BBC9-08ADAC152AE4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>STT</t>
   </si>
@@ -89,6 +89,15 @@
   </si>
   <si>
     <t xml:space="preserve">Thép phế </t>
+  </si>
+  <si>
+    <t>Ngày</t>
+  </si>
+  <si>
+    <t>Ca</t>
+  </si>
+  <si>
+    <t>Kíp</t>
   </si>
 </sst>
 </file>
@@ -299,6 +308,15 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -331,15 +349,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -370,7 +379,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>810586</xdr:colOff>
+      <xdr:colOff>497622</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>230601</xdr:rowOff>
     </xdr:to>
@@ -810,136 +819,172 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDCCEA64-4A42-45AE-9C60-18319983E285}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="15" style="3" customWidth="1"/>
-    <col min="5" max="5" width="18" style="3" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" style="3" customWidth="1"/>
-    <col min="8" max="8" width="11" style="3" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="3"/>
+    <col min="2" max="2" width="18" style="3" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="15" style="3" customWidth="1"/>
+    <col min="8" max="8" width="18" style="3" customWidth="1"/>
+    <col min="9" max="9" width="11.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="3" customWidth="1"/>
+    <col min="11" max="11" width="11" style="3" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="14" t="s">
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
-    <row r="2" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
     </row>
-    <row r="3" spans="1:9" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="4"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="4"/>
     </row>
-    <row r="4" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="5"/>
+    <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="5"/>
     </row>
-    <row r="5" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="5"/>
+    <row r="5" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="5"/>
     </row>
-    <row r="6" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+    <row r="6" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="F6" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="G6" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="23"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="24"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="13"/>
     </row>
-    <row r="7" spans="1:9" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="19"/>
-      <c r="B7" s="20"/>
+    <row r="7" spans="1:12" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
       <c r="C7" s="22"/>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="24"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="13"/>
     </row>
-    <row r="8" spans="1:9" s="11" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" s="11" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="12"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="12"/>
     </row>
-    <row r="9" spans="1:9" ht="16.5" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:9" ht="16.5" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:9" ht="16.5" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:9" ht="16.5" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:9" ht="16.5" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:9" ht="16.5" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:9" ht="16.5" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:12" ht="16.5" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:12" ht="16.5" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:12" ht="16.5" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:12" ht="16.5" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:12" ht="16.5" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:12" ht="16.5" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:12" ht="16.5" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="D1:E3"/>
-    <mergeCell ref="F1:H3"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:G5"/>
+  <mergeCells count="11">
+    <mergeCell ref="G1:H3"/>
+    <mergeCell ref="I1:K3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A5:J5"/>
     <mergeCell ref="A6:A7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:H6"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D6:D7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>